<commit_message>
Clarify card effects and support custom PNG illustrations
</commit_message>
<xml_diff>
--- a/design/editable/card-edit-review.xlsx
+++ b/design/editable/card-edit-review.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>PEAK target: 2.6.b. Source: design/cards.json, mod 0.6.0. All 64 cards are included. See card-edit-review.xlsx for your submitted requests and their implementation status.</t>
+          <t>PEAK target: 2.6.b. Source: design/cards.json, mod 0.6.1. All 64 cards are included. See card-edit-review.xlsx for your submitted requests and their implementation status.</t>
         </is>
       </c>
     </row>
@@ -550,46 +550,70 @@
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Current implementation</t>
+          <t>Ability key placeholder</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Notes flag known limitations. Current code shows the actual modifiers, ability handler and parameters. Existing Enabled settings are preserved during upgrade.</t>
+          <t>Keep {key} in manual card text: the game replaces it with your configured binding. Defaults: Nic of Time V, Discount Cure-All K, Bootleg Scoutmaster Bugle B, Budget Checkpoint Flag N.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Numbers in the code</t>
+          <t>Your own images</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Multiplier 0.8 = 20% less, 1.3 = 30% more. Stamina/status amounts 0.1 = 10 game units; cooldowns/delays are seconds, radii metres, chance 0.65 = 65%.</t>
+          <t>Save &lt;Key&gt;.png in art/cards beside CampfireCards.dll. See card-image-map.csv and docs/card-images.md. Restart PEAK after changing images.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>New ideas</t>
+          <t>Current implementation</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Use New ideas for new card concepts. See docs/effect-feasibility.md for supported effects and what still needs a playtest.</t>
+          <t>Notes flag known limitations. Current code shows the actual modifiers, ability handler and parameters. Existing Enabled settings are preserved during upgrade.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
+          <t>Numbers in the code</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Multiplier 0.8 = 20% less, 1.3 = 30% more. Stamina/status amounts 0.1 = 10 game units; cooldowns/delays are seconds, radii metres, chance 0.65 = 65%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>New ideas</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Use New ideas for new card concepts. See docs/effect-feasibility.md for supported effects and what still needs a playtest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
           <t>Return the file</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Save as .xlsx and send it back. CSV is also provided for Excel, Sheets, LibreOffice or a text editor.</t>
         </is>
@@ -722,12 +746,12 @@
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>Lose stamina 12% slower when climbing.</t>
+          <t>Climbing uses 12% less stamina.</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>Sprinting stamina drains 12% faster</t>
+          <t>Sprinting uses 12% more stamina.</t>
         </is>
       </c>
       <c r="K2" s="8" t="inlineStr"/>
@@ -779,7 +803,7 @@
       </c>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t>30% more fall damage.</t>
+          <t>Take 30% more fall Injury.</t>
         </is>
       </c>
       <c r="K3" s="8" t="inlineStr"/>
@@ -826,12 +850,12 @@
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>You take 35% less cold when climbing on blue ice.</t>
+          <t>Cold builds 35% slower while climbing blue ice.</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>Takes 10% longer to warm back up.</t>
+          <t>Warming up takes 10% longer.</t>
         </is>
       </c>
       <c r="K4" s="8" t="inlineStr"/>
@@ -878,12 +902,12 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>Hang still on a wall to get 4 stamina back every second.</t>
+          <t>Hang still on a wall to recover 4 stamina per second.</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t>Climbing speed is reduced by 30%</t>
+          <t>Climb 30% slower.</t>
         </is>
       </c>
       <c r="K5" s="8" t="inlineStr"/>
@@ -930,12 +954,12 @@
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>Double jump: one extra jump in mid-air. (35 second cooldown)</t>
+          <t>Jump again in mid-air for a double jump. Cooldown: 35s.</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Each double jump makes you a bit drowsy (+7.5 Drowsy).</t>
+          <t>Each double jump adds 7.5 Drowsy.</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr"/>
@@ -982,12 +1006,12 @@
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>Falls hurt 25% less.</t>
+          <t>Take 25% less fall Injury.</t>
         </is>
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>Dynamite explosions deal 3 times as much Injury.</t>
+          <t>Dynamite deals 3 times as much Injury.</t>
         </is>
       </c>
       <c r="K7" s="8" t="inlineStr"/>
@@ -1039,7 +1063,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Stamina drains 10% faster.</t>
+          <t>All stamina costs are 10% higher.</t>
         </is>
       </c>
       <c r="K8" s="8" t="inlineStr"/>
@@ -1086,12 +1110,12 @@
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>Your stamina bar is 25 longer.</t>
+          <t>Gain 25 maximum stamina.</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>You get hungry 35% faster.</t>
+          <t>Hunger builds 35% faster.</t>
         </is>
       </c>
       <c r="K9" s="8" t="inlineStr"/>
@@ -1134,7 +1158,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>Below 20 stamina, press V to restore 25 stamina (5-minute cooldown).</t>
+          <t>Press {key} below 20 stamina to recover 25. Cooldown: 5 min.</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr"/>
@@ -1182,7 +1206,7 @@
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>Sprinting tires you 15% less.</t>
+          <t>Sprinting uses 15% less stamina.</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
@@ -1234,12 +1258,12 @@
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>Stamina starts coming back 0.3 seconds sooner.</t>
+          <t>Stamina regeneration starts 0.3s sooner.</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>Stamina bar shrinks 15%</t>
+          <t>Lose 15 maximum stamina.</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr"/>
@@ -1286,15 +1310,15 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>Crouch and stay still to get stamina back 35% faster.</t>
-        </is>
-      </c>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>Nothing. You're already crouched down staying still</t>
-        </is>
-      </c>
-      <c r="K13" s="8" t="inlineStr"/>
+          <t>Crouch and stay still to recover stamina 35% faster.</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr"/>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>You're already crouched. Take a breather.</t>
+        </is>
+      </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
           <t>The humorous drawback remains text only; no added numerical penalty.</t>
@@ -1338,12 +1362,12 @@
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>You sprint 25% faster.</t>
+          <t>Sprint 25% faster.</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>Your stamina bar is 12.5 shorter.</t>
+          <t>Lose 12.5 maximum stamina.</t>
         </is>
       </c>
       <c r="K14" s="8" t="inlineStr"/>
@@ -1386,7 +1410,7 @@
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>Climb for 3 seconds straight, and the next second of climbing costs 35% less stamina.</t>
+          <t>Climb for 3s straight: climbing uses 35% less stamina for the next 1s.</t>
         </is>
       </c>
       <c r="J15" s="8" t="inlineStr"/>
@@ -1434,12 +1458,12 @@
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>Every time a campfire is lit, all your Hunger clears.</t>
+          <t>Each new campfire clears your Hunger.</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
         <is>
-          <t>You can't eat cooked food, even when a teammate feeds you.</t>
+          <t>You cannot eat cooked food, including food fed to you.</t>
         </is>
       </c>
       <c r="K16" s="8" t="inlineStr"/>
@@ -1486,12 +1510,12 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>You burn 50% slower.</t>
+          <t>Heat builds 50% slower.</t>
         </is>
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>You freeze 30% faster.</t>
+          <t>Cold builds 30% faster.</t>
         </is>
       </c>
       <c r="K17" s="8" t="inlineStr"/>
@@ -1538,12 +1562,12 @@
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>You freeze 50% slower.</t>
+          <t>Cold builds 50% slower.</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t>You burn 30% faster.</t>
+          <t>Heat builds 30% faster.</t>
         </is>
       </c>
       <c r="K18" s="8" t="inlineStr"/>
@@ -1590,12 +1614,12 @@
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>Poison builds up 35% slower.</t>
+          <t>Poison builds 35% slower.</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>You burn and freeze 25% faster.</t>
+          <t>Heat and Cold build 25% faster.</t>
         </is>
       </c>
       <c r="K19" s="8" t="inlineStr"/>
@@ -1642,7 +1666,7 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>Spores build up 35% slower.</t>
+          <t>Spores build 35% slower.</t>
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr"/>
@@ -1690,12 +1714,12 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>New thorns count 40% less.</t>
+          <t>New Thorns add 40% less status, rounded up to whole thorns.</t>
         </is>
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>Takes twice as long to remove the thorns.</t>
+          <t>Removing Thorns takes twice as long.</t>
         </is>
       </c>
       <c r="K21" s="8" t="inlineStr"/>
@@ -1742,12 +1766,12 @@
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>Once you're out of the heat, it wears off 60% faster.</t>
+          <t>Heat wears off 60% faster.</t>
         </is>
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>You burn 15% faster.</t>
+          <t>Heat builds 15% faster.</t>
         </is>
       </c>
       <c r="K22" s="8" t="inlineStr"/>
@@ -1794,12 +1818,12 @@
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>Once you're out of the cold, it wears off 60% faster.</t>
+          <t>Cold wears off 60% faster.</t>
         </is>
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>You freeze 15% faster.</t>
+          <t>Cold builds 15% faster.</t>
         </is>
       </c>
       <c r="K23" s="8" t="inlineStr"/>
@@ -1894,7 +1918,7 @@
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>Every 10 minutes while alive, gain Infinite Stamina, Invincibility or Low Gravity for 20 seconds.</t>
+          <t>Every 10 min alive: a random 20s burst of Infinite Stamina, Invincibility or Low Gravity.</t>
         </is>
       </c>
       <c r="J25" s="8" t="inlineStr"/>
@@ -1938,7 +1962,7 @@
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>Bandages and medkits heal you 25% more.</t>
+          <t>Healing items remove 25% more Injury from you.</t>
         </is>
       </c>
       <c r="J26" s="8" t="inlineStr"/>
@@ -1986,12 +2010,12 @@
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>While you have 20+ Injury, climbing and sprinting use 25% less stamina .</t>
+          <t>At 20+ Injury, climbing and sprinting use 25% less stamina.</t>
         </is>
       </c>
       <c r="J27" s="8" t="inlineStr">
         <is>
-          <t>Every injury hurts 10% more.</t>
+          <t>Take 10% more Injury.</t>
         </is>
       </c>
       <c r="K27" s="8" t="inlineStr"/>
@@ -2034,7 +2058,7 @@
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>Once per biome, press K when Poison, Spores or Drowsy reaches 35 to clear 20 of the worst one.</t>
+          <t>Press {key} at 35+ Poison, Spores or Drowsy to remove 20 from the highest. Once per biome.</t>
         </is>
       </c>
       <c r="J28" s="8" t="inlineStr"/>
@@ -2082,12 +2106,12 @@
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>Once per run, a fall that would knock you out puts you back on safe ground instead.</t>
+          <t>Once per run, cancel a fatal fall and return to safe ground.</t>
         </is>
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
-          <t>If used, prevents the next card pick.</t>
+          <t>Using it skips your next card pick.</t>
         </is>
       </c>
       <c r="K29" s="8" t="inlineStr"/>
@@ -2139,7 +2163,7 @@
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
-          <t>Every injury hurts 25% more.</t>
+          <t>Take 25% more Injury.</t>
         </is>
       </c>
       <c r="K30" s="8" t="inlineStr"/>
@@ -2177,12 +2201,12 @@
       <c r="G31" s="8" t="inlineStr"/>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>Mini  Tenacity</t>
+          <t>Mini Tenacity</t>
         </is>
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>Medical items also clear 7.5 of your worst other status.</t>
+          <t>Medical items also remove 7.5 from your highest other status.</t>
         </is>
       </c>
       <c r="J31" s="8" t="inlineStr"/>
@@ -2230,12 +2254,12 @@
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>All carried weight is cut in half, including your backpack and a carried scout.</t>
+          <t>All carried weight is 50% lighter, including backpacks and scouts.</t>
         </is>
       </c>
       <c r="J32" s="8" t="inlineStr">
         <is>
-          <t>Your third pocket is locked for the rest of the run.</t>
+          <t>Your third pocket cannot hold new items.</t>
         </is>
       </c>
       <c r="K32" s="8" t="inlineStr"/>
@@ -2282,12 +2306,12 @@
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>Items in your hands weigh 25% less.</t>
+          <t>Held items weigh 25% less.</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>Items inside your backpack weigh 10% more.</t>
+          <t>Backpack contents weigh 10% more.</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr"/>
@@ -2334,12 +2358,12 @@
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>Once per biome, the first cooked food you eat isn't used up.</t>
+          <t>Once per biome, your first cooked meal is not consumed.</t>
         </is>
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
-          <t>Uncooked food cures hunger 50% less.</t>
+          <t>Uncooked food removes 50% less Hunger.</t>
         </is>
       </c>
       <c r="K34" s="8" t="inlineStr"/>
@@ -2386,12 +2410,12 @@
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
-          <t>A Balloon Bunch appears for you at the next campfire (once per run).</t>
+          <t>Get one Balloon Bunch at the next campfire. Once per run.</t>
         </is>
       </c>
       <c r="J35" s="8" t="inlineStr">
         <is>
-          <t>Every stamina use costs 10% more.</t>
+          <t>All stamina costs are 10% higher.</t>
         </is>
       </c>
       <c r="K35" s="8" t="inlineStr"/>
@@ -2438,12 +2462,12 @@
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>Get 2 more random cards right now.</t>
+          <t>Immediately gain 2 random bonus cards.</t>
         </is>
       </c>
       <c r="J36" s="8" t="inlineStr">
         <is>
-          <t>Gain one random, permanent drawback: +15% climbing cost, +15% sprint cost, +20% Injury or +20% Hunger.</t>
+          <t>One permanent random penalty: climbing or sprinting cost +15%, Injury +20%, or Hunger buildup +20%.</t>
         </is>
       </c>
       <c r="K36" s="8" t="inlineStr"/>
@@ -2490,12 +2514,12 @@
       </c>
       <c r="I37" s="8" t="inlineStr">
         <is>
-          <t>Climbing near a teammate uses 15% less stamina for you both.</t>
+          <t>You and teammates within 6 m use 15% less climbing stamina.</t>
         </is>
       </c>
       <c r="J37" s="8" t="inlineStr">
         <is>
-          <t>Climbing alone tires you 15% more.</t>
+          <t>With no teammate within 6 m, climbing uses 15% more stamina.</t>
         </is>
       </c>
       <c r="K37" s="8" t="inlineStr"/>
@@ -2542,12 +2566,12 @@
       </c>
       <c r="I38" s="8" t="inlineStr">
         <is>
-          <t>Healing items you use on teammates heal 60% more.</t>
+          <t>Healing items used on teammates remove 60% more Injury.</t>
         </is>
       </c>
       <c r="J38" s="8" t="inlineStr">
         <is>
-          <t>Healing items you use on yourself heal 35% less.</t>
+          <t>Healing items used on yourself remove 35% less Injury.</t>
         </is>
       </c>
       <c r="K38" s="8" t="inlineStr"/>
@@ -2594,12 +2618,12 @@
       </c>
       <c r="I39" s="8" t="inlineStr">
         <is>
-          <t>Carrying a scout feels 35% lighter.</t>
+          <t>Carried scouts weigh 35% less.</t>
         </is>
       </c>
       <c r="J39" s="8" t="inlineStr">
         <is>
-          <t>While you carry a passed-out scout, their paused death timer drains at 15% of normal speed (or 15% faster if already draining).</t>
+          <t>Their paused death timer drains at 15% of normal speed. Already-active timers drain 15% faster.</t>
         </is>
       </c>
       <c r="K39" s="8" t="inlineStr"/>
@@ -2651,7 +2675,7 @@
       </c>
       <c r="J40" s="8" t="inlineStr">
         <is>
-          <t>With no teammate within 6 m, you get cold 20% faster.</t>
+          <t>With no teammate within 6 m, Cold builds 20% faster.</t>
         </is>
       </c>
       <c r="K40" s="8" t="inlineStr"/>
@@ -2694,7 +2718,7 @@
       </c>
       <c r="I41" s="8" t="inlineStr">
         <is>
-          <t>The first time you revive a teammate in each biome, you both get full extra stamina bar.</t>
+          <t>First teammate revive by feeding or statue each biome: both gain 100 yellow stamina.</t>
         </is>
       </c>
       <c r="J41" s="8" t="inlineStr"/>
@@ -2747,7 +2771,7 @@
       </c>
       <c r="J42" s="8" t="inlineStr">
         <is>
-          <t>Starting a teammate pull costs you 10 stamina (once per reach).</t>
+          <t>Starting a pull costs 10 stamina, once per continuous reach.</t>
         </is>
       </c>
       <c r="K42" s="8" t="inlineStr"/>
@@ -2794,12 +2818,12 @@
       </c>
       <c r="I43" s="8" t="inlineStr">
         <is>
-          <t>Teammates near you (6 m) get stamina back 12% faster.</t>
+          <t>Teammates within 6 m recover stamina 12% faster.</t>
         </is>
       </c>
       <c r="J43" s="8" t="inlineStr">
         <is>
-          <t>With no teammate within 6 m, every stamina use costs you 10% more.</t>
+          <t>With no teammate within 6 m, all stamina costs are 10% higher.</t>
         </is>
       </c>
       <c r="K43" s="8" t="inlineStr"/>
@@ -2851,7 +2875,7 @@
       </c>
       <c r="J44" s="8" t="inlineStr">
         <is>
-          <t>Falls hurt 40% more.</t>
+          <t>Take 40% more fall Injury.</t>
         </is>
       </c>
       <c r="K44" s="8" t="inlineStr"/>
@@ -2898,12 +2922,12 @@
       </c>
       <c r="I45" s="8" t="inlineStr">
         <is>
-          <t>Get 30 extra stamina now, and 20 more at every campfire after.</t>
+          <t>Gain 30 yellow stamina now, then 20 at each later campfire.</t>
         </is>
       </c>
       <c r="J45" s="8" t="inlineStr">
         <is>
-          <t>Get 10 Curse now, and 2 more at every campfire after.</t>
+          <t>Gain 10 Curse now, then 2 at each later campfire.</t>
         </is>
       </c>
       <c r="K45" s="8" t="inlineStr"/>
@@ -2950,12 +2974,12 @@
       </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>Everything you carry is 10% lighter. In each biome, a 65% chance of 25 extra stamina.</t>
+          <t>Inventory items weigh 10% less. Each biome: 65% chance of 25 yellow stamina.</t>
         </is>
       </c>
       <c r="J46" s="8" t="inlineStr">
         <is>
-          <t>Otherwise, you take 20 Injury.</t>
+          <t>A failed roll adds 20 Injury instead.</t>
         </is>
       </c>
       <c r="K46" s="8" t="inlineStr"/>
@@ -3002,12 +3026,12 @@
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>Once per biome, press B for 60 extra stamina.</t>
+          <t>Press {key} to gain 60 yellow stamina. Once per biome.</t>
         </is>
       </c>
       <c r="J47" s="8" t="inlineStr">
         <is>
-          <t>Using it costs you 15 Injury.</t>
+          <t>Each use adds 15 Injury.</t>
         </is>
       </c>
       <c r="K47" s="8" t="inlineStr"/>
@@ -3054,12 +3078,12 @@
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>Your stamina bar is 40 longer.</t>
+          <t>Gain 40 maximum stamina.</t>
         </is>
       </c>
       <c r="J48" s="8" t="inlineStr">
         <is>
-          <t>Every injury hurts 50% more.</t>
+          <t>Take 50% more Injury.</t>
         </is>
       </c>
       <c r="K48" s="8" t="inlineStr"/>
@@ -3106,12 +3130,12 @@
       </c>
       <c r="I49" s="8" t="inlineStr">
         <is>
-          <t>You turn to stone 35% slower.</t>
+          <t>Petrification builds 35% slower.</t>
         </is>
       </c>
       <c r="J49" s="8" t="inlineStr">
         <is>
-          <t>Fall damage hurts 15% more</t>
+          <t>Take 15% more fall Injury.</t>
         </is>
       </c>
       <c r="K49" s="8" t="inlineStr"/>
@@ -3158,12 +3182,12 @@
       </c>
       <c r="I50" s="8" t="inlineStr">
         <is>
-          <t>Give up one of your cards: your stamina bar becomes 35 longer.</t>
+          <t>Sacrifice one of your cards to gain 35 maximum stamina.</t>
         </is>
       </c>
       <c r="J50" s="8" t="inlineStr">
         <is>
-          <t>Get 5 Curse at every campfire after.</t>
+          <t>Gain 5 Curse at each later campfire.</t>
         </is>
       </c>
       <c r="K50" s="8" t="inlineStr"/>
@@ -3210,7 +3234,7 @@
       </c>
       <c r="I51" s="8" t="inlineStr">
         <is>
-          <t>Climbing never tires you, falls never hurt, and you sprint 25% faster.</t>
+          <t>Climbing costs no stamina and falls cause no Injury. Sprint 25% faster.</t>
         </is>
       </c>
       <c r="J51" s="8" t="inlineStr"/>
@@ -3341,12 +3365,12 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Lose stamina 12% slower when climbing.</t>
+          <t>Climbing uses 12% less stamina.</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>Sprinting stamina drains 12% faster</t>
+          <t>Sprinting uses 12% more stamina.</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr"/>
@@ -3389,7 +3413,7 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>30% more fall damage.</t>
+          <t>Take 30% more fall Injury.</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr"/>
@@ -3427,12 +3451,12 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>You take 35% less cold when climbing on blue ice.</t>
+          <t>Cold builds 35% slower while climbing blue ice.</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Takes 10% longer to warm back up.</t>
+          <t>Warming up takes 10% longer.</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr"/>
@@ -3470,12 +3494,12 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Hang still on a wall to get 4 stamina back every second.</t>
+          <t>Hang still on a wall to recover 4 stamina per second.</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Climbing speed is reduced by 30%</t>
+          <t>Climb 30% slower.</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
@@ -3513,12 +3537,12 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Double jump: one extra jump in mid-air. (35 second cooldown)</t>
+          <t>Jump again in mid-air for a double jump. Cooldown: 35s.</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Each double jump makes you a bit drowsy (+7.5 Drowsy).</t>
+          <t>Each double jump adds 7.5 Drowsy.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr"/>
@@ -3556,12 +3580,12 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>You climb 30% faster.</t>
+          <t>Climb 30% faster.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Climbing tires you 20% more.</t>
+          <t>Climbing uses 20% more stamina.</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
@@ -3599,12 +3623,12 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Falls hurt 25% less.</t>
+          <t>Take 25% less fall Injury.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Dynamite explosions deal 3 times as much Injury.</t>
+          <t>Dynamite deals 3 times as much Injury.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr"/>
@@ -3647,7 +3671,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Stamina drains 10% faster.</t>
+          <t>All stamina costs are 10% higher.</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
@@ -3685,12 +3709,12 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Your stamina bar is 25 longer.</t>
+          <t>Gain 25 maximum stamina.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>You get hungry 35% faster.</t>
+          <t>Hunger builds 35% faster.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr"/>
@@ -3728,7 +3752,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Below 20 stamina, press V to restore 25 stamina (5-minute cooldown).</t>
+          <t>Press {key} below 20 stamina to recover 25. Cooldown: 5 min.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr"/>
@@ -3771,7 +3795,7 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Sprinting tires you 15% less.</t>
+          <t>Sprinting uses 15% less stamina.</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -3814,12 +3838,12 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Stamina starts coming back 0.3 seconds sooner.</t>
+          <t>Stamina regeneration starts 0.3s sooner.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Stamina bar shrinks 15%</t>
+          <t>Lose 15 maximum stamina.</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
@@ -3857,15 +3881,15 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Crouch and stay still to get stamina back 35% faster.</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>Nothing. You're already crouched down staying still</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr"/>
+          <t>Crouch and stay still to recover stamina 35% faster.</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>You're already crouched. Take a breather.</t>
+        </is>
+      </c>
       <c r="J14" s="6" t="inlineStr"/>
       <c r="K14" s="4" t="inlineStr"/>
     </row>
@@ -3900,12 +3924,12 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>You sprint 25% faster.</t>
+          <t>Sprint 25% faster.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Your stamina bar is 12.5 shorter.</t>
+          <t>Lose 12.5 maximum stamina.</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
@@ -3943,7 +3967,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Climb for 3 seconds straight, and the next second of climbing costs 35% less stamina.</t>
+          <t>Climb for 3s straight: climbing uses 35% less stamina for the next 1s.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr"/>
@@ -3982,12 +4006,12 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Every time a campfire is lit, all your Hunger clears.</t>
+          <t>Each new campfire clears your Hunger.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>You can't eat cooked food, even when a teammate feeds you.</t>
+          <t>You cannot eat cooked food, including food fed to you.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
@@ -4025,12 +4049,12 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>You burn 50% slower.</t>
+          <t>Heat builds 50% slower.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>You freeze 30% faster.</t>
+          <t>Cold builds 30% faster.</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
@@ -4068,12 +4092,12 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>You freeze 50% slower.</t>
+          <t>Cold builds 50% slower.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>You burn 30% faster.</t>
+          <t>Heat builds 30% faster.</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
@@ -4111,12 +4135,12 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Poison builds up 35% slower.</t>
+          <t>Poison builds 35% slower.</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>You burn and freeze 25% faster.</t>
+          <t>Heat and Cold build 25% faster.</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
@@ -4154,7 +4178,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Spores build up 35% slower.</t>
+          <t>Spores build 35% slower.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr"/>
@@ -4201,12 +4225,12 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>New thorns count 40% less.</t>
+          <t>New Thorns add 40% less status, rounded up to whole thorns.</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>Takes twice as long to remove the thorns.</t>
+          <t>Removing Thorns takes twice as long.</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
@@ -4248,12 +4272,12 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Once you're out of the heat, it wears off 60% faster.</t>
+          <t>Heat wears off 60% faster.</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>You burn 15% faster.</t>
+          <t>Heat builds 15% faster.</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
@@ -4291,12 +4315,12 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Once you're out of the cold, it wears off 60% faster.</t>
+          <t>Cold wears off 60% faster.</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>You freeze 15% faster.</t>
+          <t>Cold builds 15% faster.</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
@@ -4377,7 +4401,7 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Every 10 minutes while alive, gain Infinite Stamina, Invincibility or Low Gravity for 20 seconds.</t>
+          <t>Every 10 min alive: a random 20s burst of Infinite Stamina, Invincibility or Low Gravity.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr"/>
@@ -4420,7 +4444,7 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Bandages and medkits heal you 25% more.</t>
+          <t>Healing items remove 25% more Injury from you.</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr"/>
@@ -4463,12 +4487,12 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>While you have 20+ Injury, climbing and sprinting use 25% less stamina .</t>
+          <t>At 20+ Injury, climbing and sprinting use 25% less stamina.</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Every injury hurts 10% more.</t>
+          <t>Take 10% more Injury.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr"/>
@@ -4506,7 +4530,7 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Once per biome, press K when Poison, Spores or Drowsy reaches 35 to clear 20 of the worst one.</t>
+          <t>Press {key} at 35+ Poison, Spores or Drowsy to remove 20 from the highest. Once per biome.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr"/>
@@ -4549,12 +4573,12 @@
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>Once per run, a fall that would knock you out puts you back on safe ground instead.</t>
+          <t>Once per run, cancel a fatal fall and return to safe ground.</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>If used, prevents the next card pick.</t>
+          <t>Using it skips your next card pick.</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
@@ -4592,7 +4616,7 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Food fills you up 20% more.</t>
+          <t>Food removes 20% more Hunger.</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr"/>
@@ -4636,7 +4660,7 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Every injury hurts 25% more.</t>
+          <t>Take 25% more Injury.</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr"/>
@@ -4669,12 +4693,12 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Mini  Tenacity</t>
+          <t>Mini Tenacity</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>Medical items also clear 7.5 of your worst other status.</t>
+          <t>Medical items also remove 7.5 from your highest other status.</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr"/>
@@ -4717,12 +4741,12 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>All carried weight is cut in half, including your backpack and a carried scout.</t>
+          <t>All carried weight is 50% lighter, including backpacks and scouts.</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>Your third pocket is locked for the rest of the run.</t>
+          <t>Your third pocket cannot hold new items.</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr"/>
@@ -4764,12 +4788,12 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>Items in your hands weigh 25% less.</t>
+          <t>Held items weigh 25% less.</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>Items inside your backpack weigh 10% more.</t>
+          <t>Backpack contents weigh 10% more.</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr"/>
@@ -4807,7 +4831,7 @@
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>The item in your hands weighs 35% less.</t>
+          <t>Held items weigh 35% less.</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr"/>
@@ -4846,12 +4870,12 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Once per biome, the first cooked food you eat isn't used up.</t>
+          <t>Once per biome, your first cooked meal is not consumed.</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>Uncooked food cures hunger 50% less.</t>
+          <t>Uncooked food removes 50% less Hunger.</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
@@ -4893,12 +4917,12 @@
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>Cooked food fills you up 50% more.</t>
+          <t>Cooked food removes 50% more Hunger.</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>Eating uncooked food poisons you a little (+7.5 Poison).</t>
+          <t>Eating cookable food raw adds 7.5 Poison.</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
@@ -4936,12 +4960,12 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>A Balloon Bunch appears for you at the next campfire (once per run).</t>
+          <t>Get one Balloon Bunch at the next campfire. Once per run.</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>Every stamina use costs 10% more.</t>
+          <t>All stamina costs are 10% higher.</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
@@ -4979,7 +5003,7 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>A free bandage appears for you at each new campfire.</t>
+          <t>Get a Bandage at each new campfire after picking this card.</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr"/>
@@ -5018,12 +5042,12 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Get 2 more random cards right now.</t>
+          <t>Immediately gain 2 random bonus cards.</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>Gain one random, permanent drawback: +15% climbing cost, +15% sprint cost, +20% Injury or +20% Hunger.</t>
+          <t>One permanent random penalty: climbing or sprinting cost +15%, Injury +20%, or Hunger buildup +20%.</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr"/>
@@ -5065,12 +5089,12 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>Climbing near a teammate uses 15% less stamina for you both.</t>
+          <t>You and teammates within 6 m use 15% less climbing stamina.</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>Climbing alone tires you 15% more.</t>
+          <t>With no teammate within 6 m, climbing uses 15% more stamina.</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr"/>
@@ -5108,12 +5132,12 @@
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>Healing items you use on teammates heal 60% more.</t>
+          <t>Healing items used on teammates remove 60% more Injury.</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Healing items you use on yourself heal 35% less.</t>
+          <t>Healing items used on yourself remove 35% less Injury.</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr"/>
@@ -5155,12 +5179,12 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>Carrying a scout feels 35% lighter.</t>
+          <t>Carried scouts weigh 35% less.</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>While you carry a passed-out scout, their paused death timer drains at 15% of normal speed (or 15% faster if already draining).</t>
+          <t>Their paused death timer drains at 15% of normal speed. Already-active timers drain 15% faster.</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr"/>
@@ -5203,7 +5227,7 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>With no teammate within 6 m, you get cold 20% faster.</t>
+          <t>With no teammate within 6 m, Cold builds 20% faster.</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr"/>
@@ -5241,7 +5265,7 @@
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>The first time you revive a teammate in each biome, you both get full extra stamina bar.</t>
+          <t>First teammate revive by feeding or statue each biome: both gain 100 yellow stamina.</t>
         </is>
       </c>
       <c r="H46" s="6" t="inlineStr"/>
@@ -5289,7 +5313,7 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>Starting a teammate pull costs you 10 stamina (once per reach).</t>
+          <t>Starting a pull costs 10 stamina, once per continuous reach.</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr"/>
@@ -5327,12 +5351,12 @@
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>Teammates near you (6 m) take 30% less injury.</t>
+          <t>Teammates within 6 m take 30% less Injury.</t>
         </is>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>You take half of what you saved them (at most 10 per hit).</t>
+          <t>You take half the prevented Injury, up to 10 per hit.</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr"/>
@@ -5370,12 +5394,12 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>Teammates near you (6 m) get stamina back 12% faster.</t>
+          <t>Teammates within 6 m recover stamina 12% faster.</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>With no teammate within 6 m, every stamina use costs you 10% more.</t>
+          <t>With no teammate within 6 m, all stamina costs are 10% higher.</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr"/>
@@ -5418,7 +5442,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>Falls hurt 40% more.</t>
+          <t>Take 40% more fall Injury.</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr"/>
@@ -5456,12 +5480,12 @@
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>Get 30 extra stamina now, and 20 more at every campfire after.</t>
+          <t>Gain 30 yellow stamina now, then 20 at each later campfire.</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>Get 10 Curse now, and 2 more at every campfire after.</t>
+          <t>Gain 10 Curse now, then 2 at each later campfire.</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr"/>
@@ -5499,12 +5523,12 @@
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>Everything you carry is 10% lighter. In each biome, a 65% chance of 25 extra stamina.</t>
+          <t>Inventory items weigh 10% less. Each biome: 65% chance of 25 yellow stamina.</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>Otherwise, you take 20 Injury.</t>
+          <t>A failed roll adds 20 Injury instead.</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr"/>
@@ -5542,12 +5566,12 @@
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>Once per biome, press B for 60 extra stamina.</t>
+          <t>Press {key} to gain 60 yellow stamina. Once per biome.</t>
         </is>
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>Using it costs you 15 Injury.</t>
+          <t>Each use adds 15 Injury.</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr"/>
@@ -5589,12 +5613,12 @@
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>Sprint for 2 seconds and you speed up 30% until you stop.</t>
+          <t>Sprint for 2s to move 30% faster until you stop.</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>Stopping after the speed-up makes you a bit drowsy (+7.5 Drowsy, at most every 30 seconds).</t>
+          <t>Stopping after a boost adds 7.5 Drowsy, at most once every 30s.</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr"/>
@@ -5632,7 +5656,7 @@
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>Falls hurt 15% less, and most of the injury only arrives 20 seconds later.</t>
+          <t>Take 25% of a fall's Injury now and 60% after 20s: 15% less in total.</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr"/>
@@ -5671,12 +5695,12 @@
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>Your stamina bar is 40 longer.</t>
+          <t>Gain 40 maximum stamina.</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>Every injury hurts 50% more.</t>
+          <t>Take 50% more Injury.</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr"/>
@@ -5714,12 +5738,12 @@
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>Without a backpack, sprint 30% faster and jump 20% higher.</t>
+          <t>Without a backpack: sprint 30% faster and jump 20% higher.</t>
         </is>
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>With a backpack, you sprint 15% slower.</t>
+          <t>With a backpack: sprint 15% slower.</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr"/>
@@ -5757,12 +5781,12 @@
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>Get 1 more random card right now (Common to Rare).</t>
+          <t>Immediately gain 1 random bonus card, Common to Rare.</t>
         </is>
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>Get 10 Curse now, and the next campfire offers you only 1 card.</t>
+          <t>Gain 10 Curse. Your next campfire offers only 1 card.</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr"/>
@@ -5800,7 +5824,7 @@
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>See food, items and luggage within 12 m, even through rock.</t>
+          <t>Mark food, items and luggage within 12 m, even through terrain.</t>
         </is>
       </c>
       <c r="H59" s="6" t="inlineStr"/>
@@ -5843,7 +5867,7 @@
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>Eating while you have 20+ Injury heals 7.5 Injury.</t>
+          <t>At 20+ Injury, eating food removes 7.5 Injury.</t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr"/>
@@ -5882,12 +5906,12 @@
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>Once per biome, press N to set an anchor. If you pass out, you wake up there.</t>
+          <t>Press {key} on flat ground: your next pass-out revives you here. Once per biome.</t>
         </is>
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>Your stamina bar is 15 shorter.</t>
+          <t>Lose 15 maximum stamina. The revival leaves 40 Injury.</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr"/>
@@ -5925,12 +5949,12 @@
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>You turn to stone 35% slower.</t>
+          <t>Petrification builds 35% slower.</t>
         </is>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>Fall damage hurts 15% more</t>
+          <t>Take 15% more fall Injury.</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr"/>
@@ -5968,12 +5992,12 @@
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>Give up one of your cards: your stamina bar becomes 35 longer.</t>
+          <t>Sacrifice one of your cards to gain 35 maximum stamina.</t>
         </is>
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>Get 5 Curse at every campfire after.</t>
+          <t>Gain 5 Curse at each later campfire.</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr"/>
@@ -6011,7 +6035,7 @@
       </c>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>Climbing never tires you, falls never hurt, and you sprint 25% faster.</t>
+          <t>Climbing costs no stamina and falls cause no Injury. Sprint 25% faster.</t>
         </is>
       </c>
       <c r="H64" s="6" t="inlineStr"/>
@@ -6054,7 +6078,7 @@
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>Everyone within 15 m of you (you too) gets a stamina bar 35 longer and takes 60% less injury and statuses. Once per biome, the first scout nearby who passes out is revived.</t>
+          <t>You and scouts within 15 m: maximum stamina +35; Injury and status buildup -60%. Share 1 auto-revive per biome.</t>
         </is>
       </c>
       <c r="H65" s="6" t="inlineStr"/>

</xml_diff>